<commit_message>
refactor: simplify test case structure by using multi-line strings for steps and expected results instead of multiple columns
</commit_message>
<xml_diff>
--- a/tools/e2e/test-cases-template.xlsx
+++ b/tools/e2e/test-cases-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:K6"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -407,23 +407,10 @@
     <col min="5" max="5" width="40.83203125" customWidth="1"/>
     <col min="6" max="6" width="50.83203125" customWidth="1"/>
     <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
-    <col min="9" max="9" width="50.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
-    <col min="11" max="11" width="50.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="50.83203125" customWidth="1"/>
-    <col min="14" max="14" width="50.83203125" customWidth="1"/>
-    <col min="15" max="15" width="50.83203125" customWidth="1"/>
-    <col min="16" max="16" width="50.83203125" customWidth="1"/>
-    <col min="17" max="17" width="50.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1"/>
-    <col min="19" max="19" width="40.83203125" customWidth="1"/>
-    <col min="20" max="20" width="40.83203125" customWidth="1"/>
-    <col min="21" max="21" width="40.83203125" customWidth="1"/>
-    <col min="22" max="22" width="40.83203125" customWidth="1"/>
-    <col min="23" max="23" width="10.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="80.83203125" customWidth="1"/>
+    <col min="9" max="9" width="80.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,58 +436,19 @@
         <v>Prerequisites</v>
       </c>
       <c r="H1" t="str">
-        <v>Step 1</v>
+        <v>Steps</v>
       </c>
       <c r="I1" t="str">
-        <v>Step 2</v>
+        <v>Expected Results</v>
       </c>
       <c r="J1" t="str">
-        <v>Step 3</v>
+        <v>Priority</v>
       </c>
       <c r="K1" t="str">
-        <v>Step 4</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Step 5</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Step 6</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Step 7</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Step 8</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Step 9</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Step 10</v>
-      </c>
-      <c r="R1" t="str">
-        <v>Expected Result 1</v>
-      </c>
-      <c r="S1" t="str">
-        <v>Expected Result 2</v>
-      </c>
-      <c r="T1" t="str">
-        <v>Expected Result 3</v>
-      </c>
-      <c r="U1" t="str">
-        <v>Expected Result 4</v>
-      </c>
-      <c r="V1" t="str">
-        <v>Expected Result 5</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Priority</v>
-      </c>
-      <c r="X1" t="str">
         <v>Status</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>TC-QA-001</v>
       </c>
@@ -522,59 +470,27 @@
       <c r="G2" t="str">
         <v>email=admin@example.com; password=admin123</v>
       </c>
-      <c r="H2" t="str">
-        <v>Navigate to the login page</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Wait for the page to fully load</v>
+      <c r="H2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to the login page
+2. Wait for the page to fully load
+3. Verify the quick access login buttons are visible below the login form
+4. Verify there are demo account buttons rendered by the extension slot</v>
+      </c>
+      <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">- Login page loads with the standard login form
+- Quick access buttons section is visible below the form
+- At least one demo account button is displayed
+- Buttons show user names (e.g., Admin User)
+- Extension slot renders without errors</v>
       </c>
       <c r="J2" t="str">
-        <v>Verify the quick access login buttons are visible below the login form</v>
+        <v>High</v>
       </c>
       <c r="K2" t="str">
-        <v>Verify there are demo account buttons rendered by the extension slot</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v>Login page loads with the standard login form</v>
-      </c>
-      <c r="S2" t="str">
-        <v>Quick access buttons section is visible below the form</v>
-      </c>
-      <c r="T2" t="str">
-        <v>At least one demo account button is displayed</v>
-      </c>
-      <c r="U2" t="str">
-        <v>Buttons show user names (e.g., Admin User)</v>
-      </c>
-      <c r="V2" t="str">
-        <v>Extension slot renders without errors</v>
-      </c>
-      <c r="W2" t="str">
-        <v>High</v>
-      </c>
-      <c r="X2" t="str">
         <v>Automated</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>TC-QA-002</v>
       </c>
@@ -596,59 +512,26 @@
       <c r="G3" t="str">
         <v>email=admin@example.com; password=admin123</v>
       </c>
-      <c r="H3" t="str">
-        <v>Navigate to the login page</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Click the Admin User quick access demo account button</v>
+      <c r="H3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to the login page
+2. Click the Admin User quick access demo account button
+3. Wait for the page to redirect after login
+4. Verify the user is logged in and sees the dashboard</v>
+      </c>
+      <c r="I3" t="str" xml:space="preserve">
+        <v xml:space="preserve">- Clicking the button initiates login
+- Page redirects to dashboard or home
+- User profile shows Admin User
+- No error messages displayed</v>
       </c>
       <c r="J3" t="str">
-        <v>Wait for the page to redirect after login</v>
+        <v>High</v>
       </c>
       <c r="K3" t="str">
-        <v>Verify the user is logged in and sees the dashboard</v>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
-        <v>Clicking the button initiates login</v>
-      </c>
-      <c r="S3" t="str">
-        <v>Page redirects to dashboard or home</v>
-      </c>
-      <c r="T3" t="str">
-        <v>User profile shows Admin User</v>
-      </c>
-      <c r="U3" t="str">
-        <v>No error messages displayed</v>
-      </c>
-      <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v>High</v>
-      </c>
-      <c r="X3" t="str">
         <v>Automated</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>TC-API-001</v>
       </c>
@@ -670,59 +553,27 @@
       <c r="G4" t="str">
         <v>email=admin@example.com; password=admin123</v>
       </c>
-      <c r="H4" t="str">
-        <v>Send POST request to /api/auth/login with email and password from prerequisites</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Assert response status is 200</v>
+      <c r="H4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Send POST request to /api/auth/login with email and password from prerequisites
+2. Assert response status is 200
+3. Assert response body contains "accessToken" field
+4. Use the token to send GET request to /api/auth/profile
+5. Assert response status is 200
+6. Assert response body field "user.email" equals "admin@example.com"</v>
+      </c>
+      <c r="I4" t="str" xml:space="preserve">
+        <v xml:space="preserve">- Login returns HTTP 200 with a JWT token
+- Profile endpoint accepts the token and returns user data
+- Email in profile matches the login credential</v>
       </c>
       <c r="J4" t="str">
-        <v>Assert response body contains "accessToken" field</v>
+        <v>High</v>
       </c>
       <c r="K4" t="str">
-        <v>Use the token to send GET request to /api/auth/profile</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Assert response status is 200</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Assert response body field "user.email" equals "admin@example.com"</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
-      </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
-        <v>Login returns HTTP 200 with a JWT token</v>
-      </c>
-      <c r="S4" t="str">
-        <v>Profile endpoint accepts the token and returns user data</v>
-      </c>
-      <c r="T4" t="str">
-        <v>Email in profile matches the login credential</v>
-      </c>
-      <c r="U4" t="str">
-        <v/>
-      </c>
-      <c r="V4" t="str">
-        <v/>
-      </c>
-      <c r="W4" t="str">
-        <v>High</v>
-      </c>
-      <c r="X4" t="str">
         <v>Automated</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
         <v>TC-API-002</v>
       </c>
@@ -744,59 +595,24 @@
       <c r="G5" t="str">
         <v>email=admin@example.com; password=wrongpassword</v>
       </c>
-      <c r="H5" t="str">
-        <v>Send POST request to /api/auth/login with email and wrong password</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Assert response status is 401</v>
+      <c r="H5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Send POST request to /api/auth/login with email and wrong password
+2. Assert response status is 401
+3. Assert response body contains error message</v>
+      </c>
+      <c r="I5" t="str" xml:space="preserve">
+        <v xml:space="preserve">- Login returns HTTP 401 Unauthorized
+- Response body contains an error description
+- No token is returned</v>
       </c>
       <c r="J5" t="str">
-        <v>Assert response body contains error message</v>
+        <v>High</v>
       </c>
       <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-      <c r="N5" t="str">
-        <v/>
-      </c>
-      <c r="O5" t="str">
-        <v/>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
-        <v/>
-      </c>
-      <c r="R5" t="str">
-        <v>Login returns HTTP 401 Unauthorized</v>
-      </c>
-      <c r="S5" t="str">
-        <v>Response body contains an error description</v>
-      </c>
-      <c r="T5" t="str">
-        <v>No token is returned</v>
-      </c>
-      <c r="U5" t="str">
-        <v/>
-      </c>
-      <c r="V5" t="str">
-        <v/>
-      </c>
-      <c r="W5" t="str">
-        <v>High</v>
-      </c>
-      <c r="X5" t="str">
         <v>Ready</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>TC-SYS-001</v>
       </c>
@@ -818,61 +634,31 @@
       <c r="G6" t="str">
         <v>email=admin@example.com; password=admin123</v>
       </c>
-      <c r="H6" t="str">
-        <v>Send POST request to /api/auth/login to get JWT token</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Navigate to the profile page in the browser</v>
+      <c r="H6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Send POST request to /api/auth/login to get JWT token
+2. Navigate to the profile page in the browser
+3. Verify the profile page shows the current user name
+4. Update the display name field to "Test Admin"
+5. Click the Save button
+6. Send GET request to /api/auth/profile to verify the change
+7. Assert response body field "user.display_name" equals "Test Admin"</v>
+      </c>
+      <c r="I6" t="str" xml:space="preserve">
+        <v xml:space="preserve">- Login API returns valid token
+- Profile page loads with user data
+- Name update saves successfully
+- API confirms the updated name</v>
       </c>
       <c r="J6" t="str">
-        <v>Verify the profile page shows the current user name</v>
+        <v>Medium</v>
       </c>
       <c r="K6" t="str">
-        <v>Update the display name field to "Test Admin"</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Click the Save button</v>
-      </c>
-      <c r="M6" t="str">
-        <v>Send GET request to /api/auth/profile to verify the change</v>
-      </c>
-      <c r="N6" t="str">
-        <v>Assert response body field "user.display_name" equals "Test Admin"</v>
-      </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v/>
-      </c>
-      <c r="R6" t="str">
-        <v>Login API returns valid token</v>
-      </c>
-      <c r="S6" t="str">
-        <v>Profile page loads with user data</v>
-      </c>
-      <c r="T6" t="str">
-        <v>Name update saves successfully</v>
-      </c>
-      <c r="U6" t="str">
-        <v>API confirms the updated name</v>
-      </c>
-      <c r="V6" t="str">
-        <v/>
-      </c>
-      <c r="W6" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="X6" t="str">
         <v>Draft</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1016,35 +802,35 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>H-Q</v>
+        <v>H</v>
       </c>
       <c r="B12" t="str">
-        <v>Step 1-10</v>
+        <v>Steps</v>
       </c>
       <c r="C12" t="str">
-        <v>Yes (1+)</v>
+        <v>Yes</v>
       </c>
       <c r="D12" t="str">
-        <v>Test steps in natural English — empty cells are ignored</v>
+        <v>Test steps in natural English, separated by newlines within the cell. You can use Alt+Enter (or Cmd+Option+Enter on Mac) to add a new line in Excel.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>R-V</v>
+        <v>I</v>
       </c>
       <c r="B13" t="str">
-        <v>Expected Result 1-5</v>
+        <v>Expected Results</v>
       </c>
       <c r="C13" t="str">
         <v>No</v>
       </c>
       <c r="D13" t="str">
-        <v>Acceptance criteria — empty cells are ignored</v>
+        <v>Acceptance criteria, separated by newlines within the cell.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>W</v>
+        <v>J</v>
       </c>
       <c r="B14" t="str">
         <v>Priority</v>
@@ -1058,7 +844,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>X</v>
+        <v>K</v>
       </c>
       <c r="B15" t="str">
         <v>Status</v>

</xml_diff>

<commit_message>
test(e2e): update E2E tests, executor outputs, and scripts
</commit_message>
<xml_diff>
--- a/tools/e2e/test-cases-template.xlsx
+++ b/tools/e2e/test-cases-template.xlsx
@@ -929,7 +929,7 @@
         <v/>
       </c>
       <c r="D23" t="str">
-        <v>node tools/e2e/excel-to-md.js test-cases.xlsx --dry-run</v>
+        <v>node tools/e2e/excelToMd.js test-cases.xlsx --dry-run</v>
       </c>
     </row>
     <row r="24">
@@ -943,7 +943,7 @@
         <v/>
       </c>
       <c r="D24" t="str">
-        <v>node tools/e2e/excel-to-md.js test-cases.xlsx</v>
+        <v>node tools/e2e/excelToMd.js test-cases.xlsx</v>
       </c>
     </row>
     <row r="25">
@@ -957,7 +957,7 @@
         <v/>
       </c>
       <c r="D25" t="str">
-        <v>node tools/e2e/excel-to-md.js test-cases.xlsx --force</v>
+        <v>node tools/e2e/excelToMd.js test-cases.xlsx --force</v>
       </c>
     </row>
   </sheetData>

</xml_diff>